<commit_message>
tests pass 5 rem skips
</commit_message>
<xml_diff>
--- a/examples/ml_results/ml_results_example.xlsx
+++ b/examples/ml_results/ml_results_example.xlsx
@@ -300,7 +300,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetData>
+  <sheetData>
     <x:row r="1">
       <x:c r="A1" t="s">
         <x:v>0</x:v>
@@ -597,13 +597,13 @@
         <x:v>3.3</x:v>
       </x:c>
     </x:row>
-  </x:sheetData>
+  </sheetData>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetData>
+  <sheetData>
     <x:row r="1">
       <x:c r="A1" t="s">
         <x:v>20</x:v>
@@ -865,13 +865,13 @@
         <x:f>=B13*1.5/(C13-50)</x:f>
       </x:c>
     </x:row>
-  </x:sheetData>
+  </sheetData>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetData>
+  <sheetData>
     <x:row r="1">
       <x:c r="A1" t="s">
         <x:v>28</x:v>
@@ -1107,13 +1107,13 @@
         <x:f>=C12-B12</x:f>
       </x:c>
     </x:row>
-  </x:sheetData>
+  </sheetData>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetData>
+  <sheetData>
     <x:row r="1">
       <x:c r="A1" t="s">
         <x:v>36</x:v>
@@ -1353,6 +1353,6 @@
         <x:f>=F11/G11</x:f>
       </x:c>
     </x:row>
-  </x:sheetData>
+  </sheetData>
 </x:worksheet>
 </file>
</xml_diff>